<commit_message>
Record LB for exp030 and exp031 (new best: private 0.41990, public 0.42184)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/experiments_summary.xlsx
+++ b/experiments_summary.xlsx
@@ -14,7 +14,7 @@
     <sheet name="CV と LB" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'実験一覧'!$A$1:$O$34</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'実験一覧'!$A$1:$O$38</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -321,12 +321,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'CV と LB'!$A$2:$A$23</f>
+              <f>'CV と LB'!$A$2:$A$25</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'CV と LB'!$B$2:$B$23</f>
+              <f>'CV と LB'!$B$2:$B$25</f>
             </numRef>
           </val>
         </ser>
@@ -353,12 +353,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'CV と LB'!$A$2:$A$23</f>
+              <f>'CV と LB'!$A$2:$A$25</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'CV と LB'!$C$2:$C$23</f>
+              <f>'CV と LB'!$C$2:$C$25</f>
             </numRef>
           </val>
         </ser>
@@ -739,7 +739,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Home Depot Product Search Relevance：実験の振り返り（exp001〜exp029）</t>
+          <t>Home Depot Product Search Relevance：実験の振り返り（exp001〜exp031）</t>
         </is>
       </c>
     </row>
@@ -763,7 +763,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>2026-10-13 〜 2026-10-27</t>
+          <t>2026-10-13 〜 2026-10-28</t>
         </is>
       </c>
     </row>
@@ -775,7 +775,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>exp029_all：LightGBM 単体（全部の列）。CV 0.41812 / Private LB 0.42011 / Public LB 0.42207</t>
+          <t>exp031_all：LightGBM 単体（全部の列）。CV 0.41743 / Private LB 0.41990 / Public LB 0.42184</t>
         </is>
       </c>
     </row>
@@ -787,7 +787,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>exp001：CV 0.50579 / Private LB 0.50782（ベストまで −0.0877）</t>
+          <t>exp001：CV 0.50579 / Private LB 0.50782（ベストまで −0.0879）</t>
         </is>
       </c>
     </row>
@@ -799,7 +799,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>前処理（正規化・SymSpell・ステミング）→ TF-IDF・BM25・単語一致・文字 n-gram・ブランド・属性値 → 埋め込み（mxbai-embed-large）→ 学習前の cross-encoder（mxbai-rerank-base）→ ファインチューニングした cross-encoder 5 種（bge-reranker-base ×2、v2-m3 ×2（種の平均）、DeBERTa ×1）→ 同じ検索語の中での相対値 → LightGBM（Optuna で調整、lr 0.02）</t>
+          <t>前処理（正規化・SymSpell・ステミング）→ TF-IDF・BM25・単語一致・文字 n-gram・ブランド・属性値 → 埋め込み（mxbai-embed-large）→ 学習前の cross-encoder（mxbai-rerank-base）→ ファインチューニングした cross-encoder 6 種（bge-reranker-base ×2、v2-m3 ×2（種の平均）、DeBERTa ×1、ModernBERT ×1）→ 同じ検索語の中での相対値 → LightGBM（Optuna で調整、lr 0.02）</t>
         </is>
       </c>
     </row>
@@ -930,7 +930,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O42"/>
+  <dimension ref="A1:O46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3005,66 +3005,66 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="19" t="n">
+      <c r="A33" s="8" t="n">
         <v>32</v>
       </c>
-      <c r="B33" s="19" t="inlineStr">
+      <c r="B33" s="8" t="inlineStr">
         <is>
           <t>exp029_all</t>
         </is>
       </c>
-      <c r="C33" s="19" t="inlineStr">
+      <c r="C33" s="8" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
       </c>
-      <c r="D33" s="19" t="inlineStr">
+      <c r="D33" s="8" t="inlineStr">
         <is>
           <t>ファインチューニング</t>
         </is>
       </c>
-      <c r="E33" s="19" t="inlineStr">
+      <c r="E33" s="8" t="inlineStr">
         <is>
           <t>＋ ファインチューニングした DeBERTa（mxbai-rerank-base-v1、タイトル + 説明文、transformers 4.49）</t>
         </is>
       </c>
-      <c r="F33" s="19" t="inlineStr">
+      <c r="F33" s="8" t="inlineStr">
         <is>
           <t>exp026_lgb</t>
         </is>
       </c>
-      <c r="G33" s="20" t="n">
+      <c r="G33" s="9" t="n">
         <v>0.41812</v>
       </c>
-      <c r="H33" s="21" t="n">
+      <c r="H33" s="10" t="n">
         <v>0.42011</v>
       </c>
-      <c r="I33" s="21" t="n">
+      <c r="I33" s="10" t="n">
         <v>0.42207</v>
       </c>
-      <c r="J33" s="22">
+      <c r="J33" s="11">
         <f>IF(H33="","",H33-G33)</f>
         <v/>
       </c>
-      <c r="K33" s="22">
+      <c r="K33" s="11">
         <f>IF(F33="","",G33-INDEX($G:$G,MATCH(F33,$B:$B,0)))</f>
         <v/>
       </c>
-      <c r="L33" s="22">
+      <c r="L33" s="11">
         <f>IF(OR(F33="",H33=""),"",IFERROR(IF(INDEX($H:$H,MATCH(F33,$B:$B,0))="","",H33-INDEX($H:$H,MATCH(F33,$B:$B,0))),""))</f>
         <v/>
       </c>
-      <c r="M33" s="19" t="inlineStr">
-        <is>
-          <t>採用（ベスト）</t>
-        </is>
-      </c>
-      <c r="N33" s="19" t="inlineStr">
+      <c r="M33" s="8" t="inlineStr">
+        <is>
+          <t>採用</t>
+        </is>
+      </c>
+      <c r="N33" s="8" t="inlineStr">
         <is>
           <t>1.8 億で v2-m3（5.7 億）と同精度。系統の違うモデルは LB でもしっかり効く。学習は 7 時間（GPU メモリがあふれ気味）</t>
         </is>
       </c>
-      <c r="O33" s="19" t="inlineStr">
+      <c r="O33" s="8" t="inlineStr">
         <is>
           <t>output/exp029/submission_all.csv</t>
         </is>
@@ -3132,87 +3132,343 @@
         </is>
       </c>
     </row>
+    <row r="35">
+      <c r="A35" s="8" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="8" t="inlineStr">
+        <is>
+          <t>exp030_all</t>
+        </is>
+      </c>
+      <c r="C35" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="D35" s="8" t="inlineStr">
+        <is>
+          <t>ファインチューニング</t>
+        </is>
+      </c>
+      <c r="E35" s="8" t="inlineStr">
+        <is>
+          <t>＋ ファインチューニングした DeBERTa（検索語 × タイトル）</t>
+        </is>
+      </c>
+      <c r="F35" s="8" t="inlineStr">
+        <is>
+          <t>exp029_all</t>
+        </is>
+      </c>
+      <c r="G35" s="9" t="n">
+        <v>0.41776</v>
+      </c>
+      <c r="H35" s="10" t="n">
+        <v>0.41998</v>
+      </c>
+      <c r="I35" s="10" t="n">
+        <v>0.42198</v>
+      </c>
+      <c r="J35" s="11">
+        <f>IF(H35="","",H35-G35)</f>
+        <v/>
+      </c>
+      <c r="K35" s="11">
+        <f>IF(F35="","",G35-INDEX($G:$G,MATCH(F35,$B:$B,0)))</f>
+        <v/>
+      </c>
+      <c r="L35" s="11">
+        <f>IF(OR(F35="",H35=""),"",IFERROR(IF(INDEX($H:$H,MATCH(F35,$B:$B,0))="","",H35-INDEX($H:$H,MATCH(F35,$B:$B,0))),""))</f>
+        <v/>
+      </c>
+      <c r="M35" s="8" t="inlineStr">
+        <is>
+          <t>採用</t>
+        </is>
+      </c>
+      <c r="N35" s="8" t="inlineStr">
+        <is>
+          <t>LB はわずかに改善（Public −0.00009）。単独 0.43951 はタイトル版で最良。ただし DeBERTa（タイトル + 説明文）との相関 0.945 で、CV の上乗せは −0.0004 と小さい。学習は 1 時間</t>
+        </is>
+      </c>
+      <c r="O35" s="8" t="inlineStr">
+        <is>
+          <t>output/exp030/submission_all.csv</t>
+        </is>
+      </c>
+    </row>
     <row r="36">
-      <c r="B36" s="23" t="inlineStr">
+      <c r="A36" s="16" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="16" t="inlineStr">
+        <is>
+          <t>exp030_num</t>
+        </is>
+      </c>
+      <c r="C36" s="16" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="D36" s="16" t="inlineStr">
+        <is>
+          <t>特徴量選択</t>
+        </is>
+      </c>
+      <c r="E36" s="16" t="inlineStr">
+        <is>
+          <t>同上（数値の特徴量 88 列だけ、参考）</t>
+        </is>
+      </c>
+      <c r="F36" s="16" t="inlineStr">
+        <is>
+          <t>exp030_all</t>
+        </is>
+      </c>
+      <c r="G36" s="17" t="n">
+        <v>0.41521</v>
+      </c>
+      <c r="H36" s="17" t="n"/>
+      <c r="I36" s="17" t="n"/>
+      <c r="J36" s="18">
+        <f>IF(H36="","",H36-G36)</f>
+        <v/>
+      </c>
+      <c r="K36" s="18">
+        <f>IF(F36="","",G36-INDEX($G:$G,MATCH(F36,$B:$B,0)))</f>
+        <v/>
+      </c>
+      <c r="L36" s="18">
+        <f>IF(OR(F36="",H36=""),"",IFERROR(IF(INDEX($H:$H,MATCH(F36,$B:$B,0))="","",H36-INDEX($H:$H,MATCH(F36,$B:$B,0))),""))</f>
+        <v/>
+      </c>
+      <c r="M36" s="16" t="inlineStr">
+        <is>
+          <t>参考</t>
+        </is>
+      </c>
+      <c r="N36" s="16" t="inlineStr">
+        <is>
+          <t>未提出</t>
+        </is>
+      </c>
+      <c r="O36" s="16" t="inlineStr">
+        <is>
+          <t>output/exp030/submission_num.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="19" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="19" t="inlineStr">
+        <is>
+          <t>exp031_all</t>
+        </is>
+      </c>
+      <c r="C37" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="D37" s="19" t="inlineStr">
+        <is>
+          <t>ファインチューニング</t>
+        </is>
+      </c>
+      <c r="E37" s="19" t="inlineStr">
+        <is>
+          <t>exp029 ＋ ファインチューニングした ModernBERT（gte-reranker-modernbert-base、タイトル + 説明文）</t>
+        </is>
+      </c>
+      <c r="F37" s="19" t="inlineStr">
+        <is>
+          <t>exp029_all</t>
+        </is>
+      </c>
+      <c r="G37" s="20" t="n">
+        <v>0.41743</v>
+      </c>
+      <c r="H37" s="21" t="n">
+        <v>0.4199</v>
+      </c>
+      <c r="I37" s="21" t="n">
+        <v>0.42184</v>
+      </c>
+      <c r="J37" s="22">
+        <f>IF(H37="","",H37-G37)</f>
+        <v/>
+      </c>
+      <c r="K37" s="22">
+        <f>IF(F37="","",G37-INDEX($G:$G,MATCH(F37,$B:$B,0)))</f>
+        <v/>
+      </c>
+      <c r="L37" s="22">
+        <f>IF(OR(F37="",H37=""),"",IFERROR(IF(INDEX($H:$H,MATCH(F37,$B:$B,0))="","",H37-INDEX($H:$H,MATCH(F37,$B:$B,0))),""))</f>
+        <v/>
+      </c>
+      <c r="M37" s="19" t="inlineStr">
+        <is>
+          <t>採用（ベスト）</t>
+        </is>
+      </c>
+      <c r="N37" s="19" t="inlineStr">
+        <is>
+          <t>LB で Public −0.00023、新しいベスト（exp030 とは別に exp029 に加えたもの）。別系統のリランカー。単独 0.43602 は全モデルで最良（1.5 億パラメータ）。ほかとの相関 0.87〜0.93。学習は 2 時間 40 分</t>
+        </is>
+      </c>
+      <c r="O37" s="19" t="inlineStr">
+        <is>
+          <t>output/exp031/submission_all.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="16" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="16" t="inlineStr">
+        <is>
+          <t>exp031_num</t>
+        </is>
+      </c>
+      <c r="C38" s="16" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="D38" s="16" t="inlineStr">
+        <is>
+          <t>特徴量選択</t>
+        </is>
+      </c>
+      <c r="E38" s="16" t="inlineStr">
+        <is>
+          <t>同上（数値の特徴量 88 列だけ、参考）</t>
+        </is>
+      </c>
+      <c r="F38" s="16" t="inlineStr">
+        <is>
+          <t>exp031_all</t>
+        </is>
+      </c>
+      <c r="G38" s="17" t="n">
+        <v>0.41496</v>
+      </c>
+      <c r="H38" s="17" t="n"/>
+      <c r="I38" s="17" t="n"/>
+      <c r="J38" s="18">
+        <f>IF(H38="","",H38-G38)</f>
+        <v/>
+      </c>
+      <c r="K38" s="18">
+        <f>IF(F38="","",G38-INDEX($G:$G,MATCH(F38,$B:$B,0)))</f>
+        <v/>
+      </c>
+      <c r="L38" s="18">
+        <f>IF(OR(F38="",H38=""),"",IFERROR(IF(INDEX($H:$H,MATCH(F38,$B:$B,0))="","",H38-INDEX($H:$H,MATCH(F38,$B:$B,0))),""))</f>
+        <v/>
+      </c>
+      <c r="M38" s="16" t="inlineStr">
+        <is>
+          <t>参考</t>
+        </is>
+      </c>
+      <c r="N38" s="16" t="inlineStr">
+        <is>
+          <t>未提出</t>
+        </is>
+      </c>
+      <c r="O38" s="16" t="inlineStr">
+        <is>
+          <t>output/exp031/submission_num.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" s="23" t="inlineStr">
         <is>
           <t>凡例</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="B37" s="24" t="inlineStr">
-        <is>
-          <t>緑の行</t>
-        </is>
-      </c>
-      <c r="E37" s="24" t="inlineStr">
-        <is>
-          <t>現在のベスト（exp029_all）</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="B38" s="24" t="inlineStr">
-        <is>
-          <t>オレンジの行</t>
-        </is>
-      </c>
-      <c r="E38" s="24" t="inlineStr">
-        <is>
-          <t>不採用（以降の実験の土台にしていない）</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="B39" s="24" t="inlineStr">
-        <is>
-          <t>灰色の行</t>
-        </is>
-      </c>
-      <c r="E39" s="24" t="inlineStr">
-        <is>
-          <t>検証・参考のための実験</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="B40" s="24" t="inlineStr">
-        <is>
-          <t>青い数字</t>
-        </is>
-      </c>
-      <c r="E40" s="24" t="inlineStr">
-        <is>
-          <t>Kaggle に提出して得た LB（ユーザーから共有された値）。空欄は未提出、または Public LB を記録していない</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="B41" s="24" t="inlineStr">
         <is>
-          <t>LB−CV・変化の列</t>
+          <t>緑の行</t>
         </is>
       </c>
       <c r="E41" s="24" t="inlineStr">
         <is>
-          <t>数式で計算（比較対象は「比較対象」列の実験名を「実験」列から探す）。LB の変化は、両方に Private LB があるときだけ表示</t>
+          <t>現在のベスト（exp031_all）</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="B42" s="24" t="inlineStr">
         <is>
+          <t>オレンジの行</t>
+        </is>
+      </c>
+      <c r="E42" s="24" t="inlineStr">
+        <is>
+          <t>不採用（以降の実験の土台にしていない）</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" s="24" t="inlineStr">
+        <is>
+          <t>灰色の行</t>
+        </is>
+      </c>
+      <c r="E43" s="24" t="inlineStr">
+        <is>
+          <t>検証・参考のための実験</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="B44" s="24" t="inlineStr">
+        <is>
+          <t>青い数字</t>
+        </is>
+      </c>
+      <c r="E44" s="24" t="inlineStr">
+        <is>
+          <t>Kaggle に提出して得た LB（ユーザーから共有された値）。空欄は未提出、または Public LB を記録していない</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="B45" s="24" t="inlineStr">
+        <is>
+          <t>LB−CV・変化の列</t>
+        </is>
+      </c>
+      <c r="E45" s="24" t="inlineStr">
+        <is>
+          <t>数式で計算（比較対象は「比較対象」列の実験名を「実験」列から探す）。LB の変化は、両方に Private LB があるときだけ表示</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="B46" s="24" t="inlineStr">
+        <is>
           <t>CV</t>
         </is>
       </c>
-      <c r="E42" s="24" t="inlineStr">
+      <c r="E46" s="24" t="inlineStr">
         <is>
           <t>検索語単位の GroupKFold（5 分割）の RMSE。exp023〜は入れ子の CV（アンサンブル）または LightGBM 単体の OOF</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O34"/>
+  <autoFilter ref="A1:O38"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3223,7 +3479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J9"/>
+  <dimension ref="A1:J11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -3576,7 +3832,7 @@
       </c>
       <c r="D8" s="8" t="inlineStr">
         <is>
-          <t>タイトル + 説明文（256）</t>
+          <t>タイトル（128）</t>
         </is>
       </c>
       <c r="E8" s="8" t="inlineStr">
@@ -3585,66 +3841,160 @@
         </is>
       </c>
       <c r="F8" s="9" t="n">
-        <v>0.43702</v>
+        <v>0.43951</v>
       </c>
       <c r="G8" s="25" t="n"/>
       <c r="H8" s="8" t="inlineStr">
         <is>
-          <t>7 時間</t>
+          <t>1 時間</t>
         </is>
       </c>
       <c r="I8" s="8" t="inlineStr">
         <is>
-          <t>exp029</t>
+          <t>exp030</t>
         </is>
       </c>
       <c r="J8" s="8" t="inlineStr">
         <is>
-          <t>transformers 5.x では NaN。ほかのスコアとの相関 0.88〜0.92</t>
+          <t>DeBERTa（タイトル + 説明文）との相関 0.945</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
+          <t>mxbai-rerank-base-v1</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>DeBERTa-v3</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>1.8 億</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>タイトル + 説明文（256）</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>transformers 4.49 の別環境。バッチ 16 × 2</t>
+        </is>
+      </c>
+      <c r="F9" s="9" t="n">
+        <v>0.43702</v>
+      </c>
+      <c r="G9" s="25" t="n"/>
+      <c r="H9" s="8" t="inlineStr">
+        <is>
+          <t>7 時間</t>
+        </is>
+      </c>
+      <c r="I9" s="8" t="inlineStr">
+        <is>
+          <t>exp029</t>
+        </is>
+      </c>
+      <c r="J9" s="8" t="inlineStr">
+        <is>
+          <t>transformers 5.x では NaN。ほかのスコアとの相関 0.88〜0.92</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>gte-reranker-modernbert-base</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>ModernBERT</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>1.5 億</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>タイトル + 説明文（256）</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>—（.venv-gpu のまま）</t>
+        </is>
+      </c>
+      <c r="F10" s="9" t="n">
+        <v>0.43602</v>
+      </c>
+      <c r="G10" s="25" t="n">
+        <v>0.582</v>
+      </c>
+      <c r="H10" s="8" t="inlineStr">
+        <is>
+          <t>2 時間 40 分</t>
+        </is>
+      </c>
+      <c r="I10" s="8" t="inlineStr">
+        <is>
+          <t>exp031</t>
+        </is>
+      </c>
+      <c r="J10" s="8" t="inlineStr">
+        <is>
+          <t>ほかのスコアとの相関 0.87〜0.93</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
           <t>（学習前）mxbai-rerank-base-v1</t>
         </is>
       </c>
-      <c r="B9" s="8" t="inlineStr">
+      <c r="B11" s="8" t="inlineStr">
         <is>
           <t>DeBERTa-v3</t>
         </is>
       </c>
-      <c r="C9" s="8" t="inlineStr">
+      <c r="C11" s="8" t="inlineStr">
         <is>
           <t>1.8 億</t>
         </is>
       </c>
-      <c r="D9" s="8" t="inlineStr">
+      <c r="D11" s="8" t="inlineStr">
         <is>
           <t>タイトル</t>
         </is>
       </c>
-      <c r="E9" s="8" t="inlineStr">
+      <c r="E11" s="8" t="inlineStr">
         <is>
           <t>ファインチューニングなし</t>
         </is>
       </c>
-      <c r="F9" s="9" t="n"/>
-      <c r="G9" s="25" t="n">
+      <c r="F11" s="9" t="n"/>
+      <c r="G11" s="25" t="n">
         <v>0.433</v>
       </c>
-      <c r="H9" s="8" t="inlineStr">
+      <c r="H11" s="8" t="inlineStr">
         <is>
           <t>51 分（採点のみ）</t>
         </is>
       </c>
-      <c r="I9" s="8" t="inlineStr">
+      <c r="I11" s="8" t="inlineStr">
         <is>
           <t>exp014〜</t>
         </is>
       </c>
-      <c r="J9" s="8" t="inlineStr">
+      <c r="J11" s="8" t="inlineStr">
         <is>
           <t>参考</t>
         </is>
@@ -3661,7 +4011,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3827,12 +4177,12 @@
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>仮説（見た検索語のスコアの偏り）は LB で否定された。仮説は小さく試し、外れたら記録して戻す</t>
+          <t>系統の違うモデルを加える効果は、加えるほど小さくなる（DeBERTa は LB −0.0024、次の ModernBERT は −0.0002）。同じ系統で入力だけ変えた版（DeBERTa タイトル）はさらに小さい</t>
         </is>
       </c>
       <c r="C11" s="8" t="inlineStr">
         <is>
-          <t>exp028</t>
+          <t>exp029, exp030, exp031</t>
         </is>
       </c>
     </row>
@@ -3842,12 +4192,12 @@
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>Private LB を見て何度も選ぶと、test への過学習になる。採否は Public LB で判断する</t>
+          <t>仮説（見た検索語のスコアの偏り）は LB で否定された。仮説は小さく試し、外れたら記録して戻す</t>
         </is>
       </c>
       <c r="C12" s="8" t="inlineStr">
         <is>
-          <t>exp027〜</t>
+          <t>exp028</t>
         </is>
       </c>
     </row>
@@ -3857,12 +4207,12 @@
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>8GB の GPU では、単語の埋め込み層の固定・8bit AdamW・バッチの分割・bf16 予測でメモリを抑えると、大きいモデルも現実的な時間で学習できる。あふれると数倍遅くなる</t>
+          <t>Private LB を見て何度も選ぶと、test への過学習になる。採否は Public LB で判断する</t>
         </is>
       </c>
       <c r="C13" s="8" t="inlineStr">
         <is>
-          <t>exp021, exp022, exp029</t>
+          <t>exp027〜</t>
         </is>
       </c>
     </row>
@@ -3872,12 +4222,12 @@
       </c>
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>ライブラリのバージョンでモデルが学習できないことがある（DeBERTa は transformers 5.x で NaN、4.49 では学習できた）</t>
+          <t>8GB の GPU では、単語の埋め込み層の固定・8bit AdamW・バッチの分割・bf16 予測でメモリを抑えると、大きいモデルも現実的な時間で学習できる。あふれると数倍遅くなる</t>
         </is>
       </c>
       <c r="C14" s="8" t="inlineStr">
         <is>
-          <t>exp018, exp029</t>
+          <t>exp021, exp022, exp029</t>
         </is>
       </c>
     </row>
@@ -3887,10 +4237,25 @@
       </c>
       <c r="B15" s="8" t="inlineStr">
         <is>
+          <t>ライブラリのバージョンでモデルが学習できないことがある（DeBERTa は transformers 5.x で NaN、4.49 では学習できた）</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>exp018, exp029</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="8" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="8" t="inlineStr">
+        <is>
           <t>長時間の処理は、ツールの 2 時間制限を避けて独立プロセスで実行し、fold ごとに保存して途中から再開できるようにする</t>
         </is>
       </c>
-      <c r="C15" s="8" t="inlineStr">
+      <c r="C16" s="8" t="inlineStr">
         <is>
           <t>exp025, exp026, exp029</t>
         </is>
@@ -3907,7 +4272,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D25"/>
+  <dimension ref="A1:D27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -4334,8 +4699,44 @@
         <v/>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" s="26">
+        <f>実験一覧!B35</f>
+        <v/>
+      </c>
+      <c r="B24" s="27">
+        <f>実験一覧!G35</f>
+        <v/>
+      </c>
+      <c r="C24" s="27">
+        <f>実験一覧!H35</f>
+        <v/>
+      </c>
+      <c r="D24" s="28">
+        <f>C24-B24</f>
+        <v/>
+      </c>
+    </row>
     <row r="25">
-      <c r="A25" s="24" t="inlineStr">
+      <c r="A25" s="26">
+        <f>実験一覧!B37</f>
+        <v/>
+      </c>
+      <c r="B25" s="27">
+        <f>実験一覧!G37</f>
+        <v/>
+      </c>
+      <c r="C25" s="27">
+        <f>実験一覧!H37</f>
+        <v/>
+      </c>
+      <c r="D25" s="28">
+        <f>C25-B25</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="24" t="inlineStr">
         <is>
           <t>緑の文字は「実験一覧」シートへの参照。LB−CV が正なら、LB が CV より悪い</t>
         </is>

</xml_diff>

<commit_message>
Add exp032: fine-tuned Qwen3-Reranker-0.6B (LLM-based) on query x title
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/experiments_summary.xlsx
+++ b/experiments_summary.xlsx
@@ -14,7 +14,7 @@
     <sheet name="CV と LB" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'実験一覧'!$A$1:$O$38</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'実験一覧'!$A$1:$O$40</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -739,7 +739,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Home Depot Product Search Relevance：実験の振り返り（exp001〜exp031）</t>
+          <t>Home Depot Product Search Relevance：実験の振り返り（exp001〜exp032）</t>
         </is>
       </c>
     </row>
@@ -930,7 +930,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O46"/>
+  <dimension ref="A1:O48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3388,87 +3388,211 @@
         </is>
       </c>
     </row>
+    <row r="39">
+      <c r="A39" s="8" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="8" t="inlineStr">
+        <is>
+          <t>exp032_all</t>
+        </is>
+      </c>
+      <c r="C39" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="D39" s="8" t="inlineStr">
+        <is>
+          <t>ファインチューニング</t>
+        </is>
+      </c>
+      <c r="E39" s="8" t="inlineStr">
+        <is>
+          <t>exp029 ＋ ファインチューニングした Qwen3-Reranker-0.6B（LLM 系、タイトル）</t>
+        </is>
+      </c>
+      <c r="F39" s="8" t="inlineStr">
+        <is>
+          <t>exp029_all</t>
+        </is>
+      </c>
+      <c r="G39" s="9" t="n">
+        <v>0.41759</v>
+      </c>
+      <c r="H39" s="9" t="n"/>
+      <c r="I39" s="9" t="n"/>
+      <c r="J39" s="11">
+        <f>IF(H39="","",H39-G39)</f>
+        <v/>
+      </c>
+      <c r="K39" s="11">
+        <f>IF(F39="","",G39-INDEX($G:$G,MATCH(F39,$B:$B,0)))</f>
+        <v/>
+      </c>
+      <c r="L39" s="11">
+        <f>IF(OR(F39="",H39=""),"",IFERROR(IF(INDEX($H:$H,MATCH(F39,$B:$B,0))="","",H39-INDEX($H:$H,MATCH(F39,$B:$B,0))),""))</f>
+        <v/>
+      </c>
+      <c r="M39" s="8" t="inlineStr">
+        <is>
+          <t>LB 待ち</t>
+        </is>
+      </c>
+      <c r="N39" s="8" t="inlineStr">
+        <is>
+          <t>単独 0.44286 と弱めだが、ほかとの相関が最も低い（0.86〜0.90）。モデル固有の入力の形が必要。gradient checkpointing なしではメモリがあふれ 30W に。学習は 6 時間</t>
+        </is>
+      </c>
+      <c r="O39" s="8" t="inlineStr">
+        <is>
+          <t>output/exp032/submission_all.csv</t>
+        </is>
+      </c>
+    </row>
     <row r="40">
-      <c r="B40" s="23" t="inlineStr">
+      <c r="A40" s="16" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="16" t="inlineStr">
+        <is>
+          <t>exp032_num</t>
+        </is>
+      </c>
+      <c r="C40" s="16" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="D40" s="16" t="inlineStr">
+        <is>
+          <t>特徴量選択</t>
+        </is>
+      </c>
+      <c r="E40" s="16" t="inlineStr">
+        <is>
+          <t>同上（数値の特徴量 88 列だけ、参考）</t>
+        </is>
+      </c>
+      <c r="F40" s="16" t="inlineStr">
+        <is>
+          <t>exp032_all</t>
+        </is>
+      </c>
+      <c r="G40" s="17" t="n">
+        <v>0.4151</v>
+      </c>
+      <c r="H40" s="17" t="n"/>
+      <c r="I40" s="17" t="n"/>
+      <c r="J40" s="18">
+        <f>IF(H40="","",H40-G40)</f>
+        <v/>
+      </c>
+      <c r="K40" s="18">
+        <f>IF(F40="","",G40-INDEX($G:$G,MATCH(F40,$B:$B,0)))</f>
+        <v/>
+      </c>
+      <c r="L40" s="18">
+        <f>IF(OR(F40="",H40=""),"",IFERROR(IF(INDEX($H:$H,MATCH(F40,$B:$B,0))="","",H40-INDEX($H:$H,MATCH(F40,$B:$B,0))),""))</f>
+        <v/>
+      </c>
+      <c r="M40" s="16" t="inlineStr">
+        <is>
+          <t>参考</t>
+        </is>
+      </c>
+      <c r="N40" s="16" t="inlineStr">
+        <is>
+          <t>未提出</t>
+        </is>
+      </c>
+      <c r="O40" s="16" t="inlineStr">
+        <is>
+          <t>output/exp032/submission_num.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="B42" s="23" t="inlineStr">
         <is>
           <t>凡例</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="B41" s="24" t="inlineStr">
-        <is>
-          <t>緑の行</t>
-        </is>
-      </c>
-      <c r="E41" s="24" t="inlineStr">
-        <is>
-          <t>現在のベスト（exp031_all）</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="B42" s="24" t="inlineStr">
-        <is>
-          <t>オレンジの行</t>
-        </is>
-      </c>
-      <c r="E42" s="24" t="inlineStr">
-        <is>
-          <t>不採用（以降の実験の土台にしていない）</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="B43" s="24" t="inlineStr">
         <is>
-          <t>灰色の行</t>
+          <t>緑の行</t>
         </is>
       </c>
       <c r="E43" s="24" t="inlineStr">
         <is>
-          <t>検証・参考のための実験</t>
+          <t>現在のベスト（exp031_all）</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="B44" s="24" t="inlineStr">
         <is>
-          <t>青い数字</t>
+          <t>オレンジの行</t>
         </is>
       </c>
       <c r="E44" s="24" t="inlineStr">
         <is>
-          <t>Kaggle に提出して得た LB（ユーザーから共有された値）。空欄は未提出、または Public LB を記録していない</t>
+          <t>不採用（以降の実験の土台にしていない）</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="B45" s="24" t="inlineStr">
         <is>
-          <t>LB−CV・変化の列</t>
+          <t>灰色の行</t>
         </is>
       </c>
       <c r="E45" s="24" t="inlineStr">
         <is>
-          <t>数式で計算（比較対象は「比較対象」列の実験名を「実験」列から探す）。LB の変化は、両方に Private LB があるときだけ表示</t>
+          <t>検証・参考のための実験</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="B46" s="24" t="inlineStr">
         <is>
+          <t>青い数字</t>
+        </is>
+      </c>
+      <c r="E46" s="24" t="inlineStr">
+        <is>
+          <t>Kaggle に提出して得た LB（ユーザーから共有された値）。空欄は未提出、または Public LB を記録していない</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="B47" s="24" t="inlineStr">
+        <is>
+          <t>LB−CV・変化の列</t>
+        </is>
+      </c>
+      <c r="E47" s="24" t="inlineStr">
+        <is>
+          <t>数式で計算（比較対象は「比較対象」列の実験名を「実験」列から探す）。LB の変化は、両方に Private LB があるときだけ表示</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="B48" s="24" t="inlineStr">
+        <is>
           <t>CV</t>
         </is>
       </c>
-      <c r="E46" s="24" t="inlineStr">
+      <c r="E48" s="24" t="inlineStr">
         <is>
           <t>検索語単位の GroupKFold（5 分割）の RMSE。exp023〜は入れ子の CV（アンサンブル）または LightGBM 単体の OOF</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O38"/>
+  <autoFilter ref="A1:O40"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3479,7 +3603,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J11"/>
+  <dimension ref="A1:J12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -3957,44 +4081,92 @@
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
         <is>
+          <t>Qwen3-Reranker-0.6B（seq-cls）</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>Qwen3（LLM）</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>6 億</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>タイトル（160、指示文の形で包む）</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>埋め込み層を固定 + 8bit AdamW + gradient checkpointing</t>
+        </is>
+      </c>
+      <c r="F11" s="9" t="n">
+        <v>0.44286</v>
+      </c>
+      <c r="G11" s="25" t="n">
+        <v>0.5610000000000001</v>
+      </c>
+      <c r="H11" s="8" t="inlineStr">
+        <is>
+          <t>6 時間</t>
+        </is>
+      </c>
+      <c r="I11" s="8" t="inlineStr">
+        <is>
+          <t>exp032</t>
+        </is>
+      </c>
+      <c r="J11" s="8" t="inlineStr">
+        <is>
+          <t>ほかのスコアとの相関 0.86〜0.90（最も低い）</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
           <t>（学習前）mxbai-rerank-base-v1</t>
         </is>
       </c>
-      <c r="B11" s="8" t="inlineStr">
+      <c r="B12" s="8" t="inlineStr">
         <is>
           <t>DeBERTa-v3</t>
         </is>
       </c>
-      <c r="C11" s="8" t="inlineStr">
+      <c r="C12" s="8" t="inlineStr">
         <is>
           <t>1.8 億</t>
         </is>
       </c>
-      <c r="D11" s="8" t="inlineStr">
+      <c r="D12" s="8" t="inlineStr">
         <is>
           <t>タイトル</t>
         </is>
       </c>
-      <c r="E11" s="8" t="inlineStr">
+      <c r="E12" s="8" t="inlineStr">
         <is>
           <t>ファインチューニングなし</t>
         </is>
       </c>
-      <c r="F11" s="9" t="n"/>
-      <c r="G11" s="25" t="n">
+      <c r="F12" s="9" t="n"/>
+      <c r="G12" s="25" t="n">
         <v>0.433</v>
       </c>
-      <c r="H11" s="8" t="inlineStr">
+      <c r="H12" s="8" t="inlineStr">
         <is>
           <t>51 分（採点のみ）</t>
         </is>
       </c>
-      <c r="I11" s="8" t="inlineStr">
+      <c r="I12" s="8" t="inlineStr">
         <is>
           <t>exp014〜</t>
         </is>
       </c>
-      <c r="J11" s="8" t="inlineStr">
+      <c r="J12" s="8" t="inlineStr">
         <is>
           <t>参考</t>
         </is>

</xml_diff>

<commit_message>
Add exp033 (all three new rerankers) and record LB for exp032
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/experiments_summary.xlsx
+++ b/experiments_summary.xlsx
@@ -14,7 +14,7 @@
     <sheet name="CV と LB" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'実験一覧'!$A$1:$O$40</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'実験一覧'!$A$1:$O$42</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -321,12 +321,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'CV と LB'!$A$2:$A$25</f>
+              <f>'CV と LB'!$A$2:$A$26</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'CV と LB'!$B$2:$B$25</f>
+              <f>'CV と LB'!$B$2:$B$26</f>
             </numRef>
           </val>
         </ser>
@@ -353,12 +353,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'CV と LB'!$A$2:$A$25</f>
+              <f>'CV と LB'!$A$2:$A$26</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'CV と LB'!$C$2:$C$25</f>
+              <f>'CV と LB'!$C$2:$C$26</f>
             </numRef>
           </val>
         </ser>
@@ -739,7 +739,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Home Depot Product Search Relevance：実験の振り返り（exp001〜exp032）</t>
+          <t>Home Depot Product Search Relevance：実験の振り返り（exp001〜exp033）</t>
         </is>
       </c>
     </row>
@@ -930,7 +930,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O48"/>
+  <dimension ref="A1:O50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3420,8 +3420,12 @@
       <c r="G39" s="9" t="n">
         <v>0.41759</v>
       </c>
-      <c r="H39" s="9" t="n"/>
-      <c r="I39" s="9" t="n"/>
+      <c r="H39" s="10" t="n">
+        <v>0.42004</v>
+      </c>
+      <c r="I39" s="10" t="n">
+        <v>0.42201</v>
+      </c>
       <c r="J39" s="11">
         <f>IF(H39="","",H39-G39)</f>
         <v/>
@@ -3436,12 +3440,12 @@
       </c>
       <c r="M39" s="8" t="inlineStr">
         <is>
-          <t>LB 待ち</t>
+          <t>採用</t>
         </is>
       </c>
       <c r="N39" s="8" t="inlineStr">
         <is>
-          <t>単独 0.44286 と弱めだが、ほかとの相関が最も低い（0.86〜0.90）。モデル固有の入力の形が必要。gradient checkpointing なしではメモリがあふれ 30W に。学習は 6 時間</t>
+          <t>LB はごくわずかに改善（Public −0.00006）。CV の改善ほど LB には効かず。単独 0.44286 と弱めだが、ほかとの相関が最も低い（0.86〜0.90）。モデル固有の入力の形が必要。gradient checkpointing なしではメモリがあふれ 30W に。学習は 6 時間</t>
         </is>
       </c>
       <c r="O39" s="8" t="inlineStr">
@@ -3512,87 +3516,211 @@
         </is>
       </c>
     </row>
+    <row r="41">
+      <c r="A41" s="8" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="8" t="inlineStr">
+        <is>
+          <t>exp033_all</t>
+        </is>
+      </c>
+      <c r="C41" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="D41" s="8" t="inlineStr">
+        <is>
+          <t>ファインチューニング</t>
+        </is>
+      </c>
+      <c r="E41" s="8" t="inlineStr">
+        <is>
+          <t>exp029 ＋ DeBERTa（タイトル）・ModernBERT・Qwen3 の 3 つを全部</t>
+        </is>
+      </c>
+      <c r="F41" s="8" t="inlineStr">
+        <is>
+          <t>exp029_all</t>
+        </is>
+      </c>
+      <c r="G41" s="9" t="n">
+        <v>0.41705</v>
+      </c>
+      <c r="H41" s="9" t="n"/>
+      <c r="I41" s="9" t="n"/>
+      <c r="J41" s="11">
+        <f>IF(H41="","",H41-G41)</f>
+        <v/>
+      </c>
+      <c r="K41" s="11">
+        <f>IF(F41="","",G41-INDEX($G:$G,MATCH(F41,$B:$B,0)))</f>
+        <v/>
+      </c>
+      <c r="L41" s="11">
+        <f>IF(OR(F41="",H41=""),"",IFERROR(IF(INDEX($H:$H,MATCH(F41,$B:$B,0))="","",H41-INDEX($H:$H,MATCH(F41,$B:$B,0))),""))</f>
+        <v/>
+      </c>
+      <c r="M41" s="8" t="inlineStr">
+        <is>
+          <t>LB 待ち</t>
+        </is>
+      </c>
+      <c r="N41" s="8" t="inlineStr">
+        <is>
+          <t>1 つずつの CV の改善の合計（0.0016）の 7 割（0.0011）。新しい学習なし</t>
+        </is>
+      </c>
+      <c r="O41" s="8" t="inlineStr">
+        <is>
+          <t>output/exp033/submission_all.csv</t>
+        </is>
+      </c>
+    </row>
     <row r="42">
-      <c r="B42" s="23" t="inlineStr">
+      <c r="A42" s="16" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="16" t="inlineStr">
+        <is>
+          <t>exp033_num</t>
+        </is>
+      </c>
+      <c r="C42" s="16" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="D42" s="16" t="inlineStr">
+        <is>
+          <t>特徴量選択</t>
+        </is>
+      </c>
+      <c r="E42" s="16" t="inlineStr">
+        <is>
+          <t>同上（数値の特徴量 96 列だけ、参考）</t>
+        </is>
+      </c>
+      <c r="F42" s="16" t="inlineStr">
+        <is>
+          <t>exp033_all</t>
+        </is>
+      </c>
+      <c r="G42" s="17" t="n">
+        <v>0.41456</v>
+      </c>
+      <c r="H42" s="17" t="n"/>
+      <c r="I42" s="17" t="n"/>
+      <c r="J42" s="18">
+        <f>IF(H42="","",H42-G42)</f>
+        <v/>
+      </c>
+      <c r="K42" s="18">
+        <f>IF(F42="","",G42-INDEX($G:$G,MATCH(F42,$B:$B,0)))</f>
+        <v/>
+      </c>
+      <c r="L42" s="18">
+        <f>IF(OR(F42="",H42=""),"",IFERROR(IF(INDEX($H:$H,MATCH(F42,$B:$B,0))="","",H42-INDEX($H:$H,MATCH(F42,$B:$B,0))),""))</f>
+        <v/>
+      </c>
+      <c r="M42" s="16" t="inlineStr">
+        <is>
+          <t>参考</t>
+        </is>
+      </c>
+      <c r="N42" s="16" t="inlineStr">
+        <is>
+          <t>未提出</t>
+        </is>
+      </c>
+      <c r="O42" s="16" t="inlineStr">
+        <is>
+          <t>output/exp033/submission_num.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="B44" s="23" t="inlineStr">
         <is>
           <t>凡例</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="B43" s="24" t="inlineStr">
-        <is>
-          <t>緑の行</t>
-        </is>
-      </c>
-      <c r="E43" s="24" t="inlineStr">
-        <is>
-          <t>現在のベスト（exp031_all）</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="B44" s="24" t="inlineStr">
-        <is>
-          <t>オレンジの行</t>
-        </is>
-      </c>
-      <c r="E44" s="24" t="inlineStr">
-        <is>
-          <t>不採用（以降の実験の土台にしていない）</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="B45" s="24" t="inlineStr">
         <is>
-          <t>灰色の行</t>
+          <t>緑の行</t>
         </is>
       </c>
       <c r="E45" s="24" t="inlineStr">
         <is>
-          <t>検証・参考のための実験</t>
+          <t>現在のベスト（exp031_all）</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="B46" s="24" t="inlineStr">
         <is>
-          <t>青い数字</t>
+          <t>オレンジの行</t>
         </is>
       </c>
       <c r="E46" s="24" t="inlineStr">
         <is>
-          <t>Kaggle に提出して得た LB（ユーザーから共有された値）。空欄は未提出、または Public LB を記録していない</t>
+          <t>不採用（以降の実験の土台にしていない）</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="B47" s="24" t="inlineStr">
         <is>
-          <t>LB−CV・変化の列</t>
+          <t>灰色の行</t>
         </is>
       </c>
       <c r="E47" s="24" t="inlineStr">
         <is>
-          <t>数式で計算（比較対象は「比較対象」列の実験名を「実験」列から探す）。LB の変化は、両方に Private LB があるときだけ表示</t>
+          <t>検証・参考のための実験</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="B48" s="24" t="inlineStr">
         <is>
+          <t>青い数字</t>
+        </is>
+      </c>
+      <c r="E48" s="24" t="inlineStr">
+        <is>
+          <t>Kaggle に提出して得た LB（ユーザーから共有された値）。空欄は未提出、または Public LB を記録していない</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="B49" s="24" t="inlineStr">
+        <is>
+          <t>LB−CV・変化の列</t>
+        </is>
+      </c>
+      <c r="E49" s="24" t="inlineStr">
+        <is>
+          <t>数式で計算（比較対象は「比較対象」列の実験名を「実験」列から探す）。LB の変化は、両方に Private LB があるときだけ表示</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="B50" s="24" t="inlineStr">
+        <is>
           <t>CV</t>
         </is>
       </c>
-      <c r="E48" s="24" t="inlineStr">
+      <c r="E50" s="24" t="inlineStr">
         <is>
           <t>検索語単位の GroupKFold（5 分割）の RMSE。exp023〜は入れ子の CV（アンサンブル）または LightGBM 単体の OOF</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O40"/>
+  <autoFilter ref="A1:O42"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4444,7 +4572,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D27"/>
+  <dimension ref="A1:D28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -4907,8 +5035,26 @@
         <v/>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="24" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="26">
+        <f>実験一覧!B39</f>
+        <v/>
+      </c>
+      <c r="B26" s="27">
+        <f>実験一覧!G39</f>
+        <v/>
+      </c>
+      <c r="C26" s="27">
+        <f>実験一覧!H39</f>
+        <v/>
+      </c>
+      <c r="D26" s="28">
+        <f>C26-B26</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="24" t="inlineStr">
         <is>
           <t>緑の文字は「実験一覧」シートへの参照。LB−CV が正なら、LB が CV より悪い</t>
         </is>

</xml_diff>

<commit_message>
Record LB for exp033 (new best: private 0.41978, public 0.42182)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/experiments_summary.xlsx
+++ b/experiments_summary.xlsx
@@ -321,12 +321,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'CV と LB'!$A$2:$A$26</f>
+              <f>'CV と LB'!$A$2:$A$27</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'CV と LB'!$B$2:$B$26</f>
+              <f>'CV と LB'!$B$2:$B$27</f>
             </numRef>
           </val>
         </ser>
@@ -353,12 +353,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'CV と LB'!$A$2:$A$26</f>
+              <f>'CV と LB'!$A$2:$A$27</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'CV と LB'!$C$2:$C$26</f>
+              <f>'CV と LB'!$C$2:$C$27</f>
             </numRef>
           </val>
         </ser>
@@ -775,7 +775,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>exp031_all：LightGBM 単体（全部の列）。CV 0.41743 / Private LB 0.41990 / Public LB 0.42184</t>
+          <t>exp033_all：LightGBM 単体（全部の列）。CV 0.41705 / Private LB 0.41978 / Public LB 0.42182</t>
         </is>
       </c>
     </row>
@@ -787,7 +787,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>exp001：CV 0.50579 / Private LB 0.50782（ベストまで −0.0879）</t>
+          <t>exp001：CV 0.50579 / Private LB 0.50782（ベストまで −0.0880）</t>
         </is>
       </c>
     </row>
@@ -799,7 +799,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>前処理（正規化・SymSpell・ステミング）→ TF-IDF・BM25・単語一致・文字 n-gram・ブランド・属性値 → 埋め込み（mxbai-embed-large）→ 学習前の cross-encoder（mxbai-rerank-base）→ ファインチューニングした cross-encoder 6 種（bge-reranker-base ×2、v2-m3 ×2（種の平均）、DeBERTa ×1、ModernBERT ×1）→ 同じ検索語の中での相対値 → LightGBM（Optuna で調整、lr 0.02）</t>
+          <t>前処理（正規化・SymSpell・ステミング）→ TF-IDF・BM25・単語一致・文字 n-gram・ブランド・属性値 → 埋め込み（mxbai-embed-large）→ 学習前の cross-encoder（mxbai-rerank-base）→ ファインチューニングした cross-encoder 8 種（bge-reranker-base ×2、v2-m3 ×2（種の平均）、DeBERTa ×2、ModernBERT ×1、Qwen3 ×1）→ 同じ検索語の中での相対値 → LightGBM（Optuna で調整、lr 0.02）</t>
         </is>
       </c>
     </row>
@@ -3261,66 +3261,66 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="19" t="n">
+      <c r="A37" s="8" t="n">
         <v>36</v>
       </c>
-      <c r="B37" s="19" t="inlineStr">
+      <c r="B37" s="8" t="inlineStr">
         <is>
           <t>exp031_all</t>
         </is>
       </c>
-      <c r="C37" s="19" t="inlineStr">
+      <c r="C37" s="8" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
       </c>
-      <c r="D37" s="19" t="inlineStr">
+      <c r="D37" s="8" t="inlineStr">
         <is>
           <t>ファインチューニング</t>
         </is>
       </c>
-      <c r="E37" s="19" t="inlineStr">
+      <c r="E37" s="8" t="inlineStr">
         <is>
           <t>exp029 ＋ ファインチューニングした ModernBERT（gte-reranker-modernbert-base、タイトル + 説明文）</t>
         </is>
       </c>
-      <c r="F37" s="19" t="inlineStr">
+      <c r="F37" s="8" t="inlineStr">
         <is>
           <t>exp029_all</t>
         </is>
       </c>
-      <c r="G37" s="20" t="n">
+      <c r="G37" s="9" t="n">
         <v>0.41743</v>
       </c>
-      <c r="H37" s="21" t="n">
+      <c r="H37" s="10" t="n">
         <v>0.4199</v>
       </c>
-      <c r="I37" s="21" t="n">
+      <c r="I37" s="10" t="n">
         <v>0.42184</v>
       </c>
-      <c r="J37" s="22">
+      <c r="J37" s="11">
         <f>IF(H37="","",H37-G37)</f>
         <v/>
       </c>
-      <c r="K37" s="22">
+      <c r="K37" s="11">
         <f>IF(F37="","",G37-INDEX($G:$G,MATCH(F37,$B:$B,0)))</f>
         <v/>
       </c>
-      <c r="L37" s="22">
+      <c r="L37" s="11">
         <f>IF(OR(F37="",H37=""),"",IFERROR(IF(INDEX($H:$H,MATCH(F37,$B:$B,0))="","",H37-INDEX($H:$H,MATCH(F37,$B:$B,0))),""))</f>
         <v/>
       </c>
-      <c r="M37" s="19" t="inlineStr">
-        <is>
-          <t>採用（ベスト）</t>
-        </is>
-      </c>
-      <c r="N37" s="19" t="inlineStr">
+      <c r="M37" s="8" t="inlineStr">
+        <is>
+          <t>採用</t>
+        </is>
+      </c>
+      <c r="N37" s="8" t="inlineStr">
         <is>
           <t>LB で Public −0.00023、新しいベスト（exp030 とは別に exp029 に加えたもの）。別系統のリランカー。単独 0.43602 は全モデルで最良（1.5 億パラメータ）。ほかとの相関 0.87〜0.93。学習は 2 時間 40 分</t>
         </is>
       </c>
-      <c r="O37" s="19" t="inlineStr">
+      <c r="O37" s="8" t="inlineStr">
         <is>
           <t>output/exp031/submission_all.csv</t>
         </is>
@@ -3517,62 +3517,66 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="8" t="n">
+      <c r="A41" s="19" t="n">
         <v>40</v>
       </c>
-      <c r="B41" s="8" t="inlineStr">
+      <c r="B41" s="19" t="inlineStr">
         <is>
           <t>exp033_all</t>
         </is>
       </c>
-      <c r="C41" s="8" t="inlineStr">
+      <c r="C41" s="19" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
       </c>
-      <c r="D41" s="8" t="inlineStr">
+      <c r="D41" s="19" t="inlineStr">
         <is>
           <t>ファインチューニング</t>
         </is>
       </c>
-      <c r="E41" s="8" t="inlineStr">
+      <c r="E41" s="19" t="inlineStr">
         <is>
           <t>exp029 ＋ DeBERTa（タイトル）・ModernBERT・Qwen3 の 3 つを全部</t>
         </is>
       </c>
-      <c r="F41" s="8" t="inlineStr">
+      <c r="F41" s="19" t="inlineStr">
         <is>
           <t>exp029_all</t>
         </is>
       </c>
-      <c r="G41" s="9" t="n">
+      <c r="G41" s="20" t="n">
         <v>0.41705</v>
       </c>
-      <c r="H41" s="9" t="n"/>
-      <c r="I41" s="9" t="n"/>
-      <c r="J41" s="11">
+      <c r="H41" s="21" t="n">
+        <v>0.41978</v>
+      </c>
+      <c r="I41" s="21" t="n">
+        <v>0.42182</v>
+      </c>
+      <c r="J41" s="22">
         <f>IF(H41="","",H41-G41)</f>
         <v/>
       </c>
-      <c r="K41" s="11">
+      <c r="K41" s="22">
         <f>IF(F41="","",G41-INDEX($G:$G,MATCH(F41,$B:$B,0)))</f>
         <v/>
       </c>
-      <c r="L41" s="11">
+      <c r="L41" s="22">
         <f>IF(OR(F41="",H41=""),"",IFERROR(IF(INDEX($H:$H,MATCH(F41,$B:$B,0))="","",H41-INDEX($H:$H,MATCH(F41,$B:$B,0))),""))</f>
         <v/>
       </c>
-      <c r="M41" s="8" t="inlineStr">
-        <is>
-          <t>LB 待ち</t>
-        </is>
-      </c>
-      <c r="N41" s="8" t="inlineStr">
-        <is>
-          <t>1 つずつの CV の改善の合計（0.0016）の 7 割（0.0011）。新しい学習なし</t>
-        </is>
-      </c>
-      <c r="O41" s="8" t="inlineStr">
+      <c r="M41" s="19" t="inlineStr">
+        <is>
+          <t>採用（ベスト）</t>
+        </is>
+      </c>
+      <c r="N41" s="19" t="inlineStr">
+        <is>
+          <t>Public で exp031 を 0.00002 上回るだけで、LB の改善のほとんどは ModernBERT による。1 つずつの CV の改善の合計（0.0016）の 7 割（0.0011）。新しい学習なし</t>
+        </is>
+      </c>
+      <c r="O41" s="19" t="inlineStr">
         <is>
           <t>output/exp033/submission_all.csv</t>
         </is>
@@ -3655,7 +3659,7 @@
       </c>
       <c r="E45" s="24" t="inlineStr">
         <is>
-          <t>現在のベスト（exp031_all）</t>
+          <t>現在のベスト（exp033_all）</t>
         </is>
       </c>
     </row>
@@ -4311,7 +4315,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4492,12 +4496,12 @@
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>仮説（見た検索語のスコアの偏り）は LB で否定された。仮説は小さく試し、外れたら記録して戻す</t>
+          <t>スコアの相関が低い（性質が違う）だけでは LB に効くとは限らない。単独で弱いモデル（Qwen3-0.6B）は CV では効いたが LB ではごくわずか。単独の強さと性質の違いの両方が要る</t>
         </is>
       </c>
       <c r="C12" s="8" t="inlineStr">
         <is>
-          <t>exp028</t>
+          <t>exp031, exp032</t>
         </is>
       </c>
     </row>
@@ -4507,12 +4511,12 @@
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>Private LB を見て何度も選ぶと、test への過学習になる。採否は Public LB で判断する</t>
+          <t>仮説（見た検索語のスコアの偏り）は LB で否定された。仮説は小さく試し、外れたら記録して戻す</t>
         </is>
       </c>
       <c r="C13" s="8" t="inlineStr">
         <is>
-          <t>exp027〜</t>
+          <t>exp028</t>
         </is>
       </c>
     </row>
@@ -4522,12 +4526,12 @@
       </c>
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>8GB の GPU では、単語の埋め込み層の固定・8bit AdamW・バッチの分割・bf16 予測でメモリを抑えると、大きいモデルも現実的な時間で学習できる。あふれると数倍遅くなる</t>
+          <t>Private LB を見て何度も選ぶと、test への過学習になる。採否は Public LB で判断する</t>
         </is>
       </c>
       <c r="C14" s="8" t="inlineStr">
         <is>
-          <t>exp021, exp022, exp029</t>
+          <t>exp027〜</t>
         </is>
       </c>
     </row>
@@ -4537,12 +4541,12 @@
       </c>
       <c r="B15" s="8" t="inlineStr">
         <is>
-          <t>ライブラリのバージョンでモデルが学習できないことがある（DeBERTa は transformers 5.x で NaN、4.49 では学習できた）</t>
+          <t>8GB の GPU では、単語の埋め込み層の固定・8bit AdamW・バッチの分割・bf16 予測でメモリを抑えると、大きいモデルも現実的な時間で学習できる。あふれると数倍遅くなる</t>
         </is>
       </c>
       <c r="C15" s="8" t="inlineStr">
         <is>
-          <t>exp018, exp029</t>
+          <t>exp021, exp022, exp029</t>
         </is>
       </c>
     </row>
@@ -4552,10 +4556,25 @@
       </c>
       <c r="B16" s="8" t="inlineStr">
         <is>
+          <t>ライブラリのバージョンでモデルが学習できないことがある（DeBERTa は transformers 5.x で NaN、4.49 では学習できた）</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>exp018, exp029</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
           <t>長時間の処理は、ツールの 2 時間制限を避けて独立プロセスで実行し、fold ごとに保存して途中から再開できるようにする</t>
         </is>
       </c>
-      <c r="C16" s="8" t="inlineStr">
+      <c r="C17" s="8" t="inlineStr">
         <is>
           <t>exp025, exp026, exp029</t>
         </is>
@@ -4572,7 +4591,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D28"/>
+  <dimension ref="A1:D29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -5053,8 +5072,26 @@
         <v/>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="24" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="26">
+        <f>実験一覧!B41</f>
+        <v/>
+      </c>
+      <c r="B27" s="27">
+        <f>実験一覧!G41</f>
+        <v/>
+      </c>
+      <c r="C27" s="27">
+        <f>実験一覧!H41</f>
+        <v/>
+      </c>
+      <c r="D27" s="28">
+        <f>C27-B27</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="24" t="inlineStr">
         <is>
           <t>緑の文字は「実験一覧」シートへの参照。LB−CV が正なら、LB が CV より悪い</t>
         </is>

</xml_diff>